<commit_message>
feat(template): ajustar posición y tamaño de imágenes en la descarga de plantilla
</commit_message>
<xml_diff>
--- a/public/inspecciones_internas.xlsx
+++ b/public/inspecciones_internas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\inspeccionessst\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D846702-3C20-4CD9-9E7F-3FDCF08769B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C82CFD84-92AF-4D66-97CA-3EE9E0854843}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28692" yWindow="2100" windowWidth="29016" windowHeight="15696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LOV" sheetId="8" r:id="rId1"/>
@@ -524,7 +524,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="25" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -672,18 +672,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="13"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
       <b/>
       <sz val="13"/>
       <color theme="1"/>
@@ -1102,7 +1090,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="129">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1185,55 +1173,55 @@
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="9" borderId="1" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1254,50 +1242,158 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="20" fontId="19" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="19" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1305,130 +1401,25 @@
     <xf numFmtId="0" fontId="18" fillId="3" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="15" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="7" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="8" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="14" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="9" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="12" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="3" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="20" fontId="22" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1464,23 +1455,8 @@
     <xf numFmtId="0" fontId="12" fillId="10" borderId="16" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="2" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -1556,7 +1532,7 @@
       <xdr:col>1</xdr:col>
       <xdr:colOff>1521</xdr:colOff>
       <xdr:row>4</xdr:row>
-      <xdr:rowOff>132489</xdr:rowOff>
+      <xdr:rowOff>136299</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -1907,35 +1883,35 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="70"/>
-      <c r="B1" s="73" t="s">
+      <c r="A1" s="65"/>
+      <c r="B1" s="68" t="s">
         <v>0</v>
       </c>
-      <c r="C1" s="74"/>
-      <c r="D1" s="74"/>
-      <c r="E1" s="74"/>
-      <c r="F1" s="74"/>
-      <c r="G1" s="74"/>
-      <c r="H1" s="74"/>
-      <c r="I1" s="74"/>
-      <c r="J1" s="74"/>
-      <c r="K1" s="75"/>
+      <c r="C1" s="69"/>
+      <c r="D1" s="69"/>
+      <c r="E1" s="69"/>
+      <c r="F1" s="69"/>
+      <c r="G1" s="69"/>
+      <c r="H1" s="69"/>
+      <c r="I1" s="69"/>
+      <c r="J1" s="69"/>
+      <c r="K1" s="70"/>
     </row>
     <row r="2" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="71"/>
-      <c r="B2" s="76"/>
-      <c r="C2" s="77"/>
-      <c r="D2" s="77"/>
-      <c r="E2" s="77"/>
-      <c r="F2" s="77"/>
-      <c r="G2" s="77"/>
-      <c r="H2" s="77"/>
-      <c r="I2" s="78"/>
-      <c r="J2" s="78"/>
-      <c r="K2" s="79"/>
+      <c r="A2" s="66"/>
+      <c r="B2" s="71"/>
+      <c r="C2" s="72"/>
+      <c r="D2" s="72"/>
+      <c r="E2" s="72"/>
+      <c r="F2" s="72"/>
+      <c r="G2" s="72"/>
+      <c r="H2" s="72"/>
+      <c r="I2" s="73"/>
+      <c r="J2" s="73"/>
+      <c r="K2" s="74"/>
     </row>
     <row r="3" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="71"/>
+      <c r="A3" s="66"/>
       <c r="B3" s="21" t="s">
         <v>1</v>
       </c>
@@ -1952,7 +1928,7 @@
       <c r="K3" s="25"/>
     </row>
     <row r="4" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="71"/>
+      <c r="A4" s="66"/>
       <c r="B4" s="21" t="s">
         <v>115</v>
       </c>
@@ -1969,7 +1945,7 @@
       <c r="K4" s="25"/>
     </row>
     <row r="5" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="71"/>
+      <c r="A5" s="66"/>
       <c r="B5" s="21" t="s">
         <v>116</v>
       </c>
@@ -1986,7 +1962,7 @@
       <c r="K5" s="25"/>
     </row>
     <row r="6" spans="1:11" ht="22.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="72"/>
+      <c r="A6" s="67"/>
       <c r="B6" s="21" t="s">
         <v>117</v>
       </c>
@@ -2016,90 +1992,90 @@
       <c r="K7" s="17"/>
     </row>
     <row r="8" spans="1:11" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="55" t="s">
+      <c r="A8" s="94" t="s">
         <v>3</v>
       </c>
-      <c r="B8" s="57"/>
-      <c r="C8" s="57"/>
-      <c r="D8" s="57"/>
-      <c r="E8" s="57"/>
-      <c r="F8" s="57"/>
-      <c r="G8" s="57"/>
-      <c r="H8" s="57"/>
-      <c r="I8" s="57"/>
-      <c r="J8" s="57"/>
-      <c r="K8" s="58"/>
+      <c r="B8" s="55"/>
+      <c r="C8" s="55"/>
+      <c r="D8" s="55"/>
+      <c r="E8" s="55"/>
+      <c r="F8" s="55"/>
+      <c r="G8" s="55"/>
+      <c r="H8" s="55"/>
+      <c r="I8" s="55"/>
+      <c r="J8" s="55"/>
+      <c r="K8" s="56"/>
     </row>
     <row r="9" spans="1:11" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="56"/>
-      <c r="B9" s="59"/>
-      <c r="C9" s="59"/>
-      <c r="D9" s="59"/>
-      <c r="E9" s="59"/>
-      <c r="F9" s="59"/>
-      <c r="G9" s="59"/>
-      <c r="H9" s="59"/>
-      <c r="I9" s="59"/>
-      <c r="J9" s="59"/>
-      <c r="K9" s="60"/>
+      <c r="A9" s="95"/>
+      <c r="B9" s="57"/>
+      <c r="C9" s="57"/>
+      <c r="D9" s="57"/>
+      <c r="E9" s="57"/>
+      <c r="F9" s="57"/>
+      <c r="G9" s="57"/>
+      <c r="H9" s="57"/>
+      <c r="I9" s="57"/>
+      <c r="J9" s="57"/>
+      <c r="K9" s="58"/>
     </row>
     <row r="10" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="66" t="s">
+      <c r="A10" s="77" t="s">
         <v>4</v>
       </c>
-      <c r="B10" s="67"/>
-      <c r="C10" s="67"/>
-      <c r="D10" s="67"/>
-      <c r="E10" s="67"/>
-      <c r="F10" s="67"/>
-      <c r="G10" s="67"/>
-      <c r="H10" s="67"/>
-      <c r="I10" s="67"/>
-      <c r="J10" s="67"/>
-      <c r="K10" s="82"/>
+      <c r="B10" s="78"/>
+      <c r="C10" s="78"/>
+      <c r="D10" s="78"/>
+      <c r="E10" s="78"/>
+      <c r="F10" s="78"/>
+      <c r="G10" s="78"/>
+      <c r="H10" s="78"/>
+      <c r="I10" s="78"/>
+      <c r="J10" s="78"/>
+      <c r="K10" s="79"/>
     </row>
     <row r="11" spans="1:11" ht="45" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="65" t="s">
+      <c r="A11" s="63" t="s">
         <v>5</v>
       </c>
-      <c r="B11" s="97"/>
-      <c r="C11" s="97"/>
-      <c r="D11" s="65" t="s">
+      <c r="B11" s="64"/>
+      <c r="C11" s="64"/>
+      <c r="D11" s="63" t="s">
         <v>6</v>
       </c>
-      <c r="E11" s="65"/>
-      <c r="F11" s="65" t="s">
+      <c r="E11" s="63"/>
+      <c r="F11" s="63" t="s">
         <v>7</v>
       </c>
-      <c r="G11" s="65"/>
-      <c r="H11" s="65"/>
-      <c r="I11" s="63" t="s">
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="61" t="s">
         <v>8</v>
       </c>
-      <c r="J11" s="63"/>
-      <c r="K11" s="32" t="s">
+      <c r="J11" s="61"/>
+      <c r="K11" s="30" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="12" spans="1:11" ht="35.549999999999997" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="64" t="s">
+      <c r="A12" s="62" t="s">
         <v>111</v>
       </c>
-      <c r="B12" s="64"/>
-      <c r="C12" s="64"/>
-      <c r="D12" s="64">
+      <c r="B12" s="62"/>
+      <c r="C12" s="62"/>
+      <c r="D12" s="62">
         <v>20602872760</v>
       </c>
-      <c r="E12" s="64"/>
-      <c r="F12" s="64" t="s">
+      <c r="E12" s="62"/>
+      <c r="F12" s="62" t="s">
         <v>112</v>
       </c>
-      <c r="G12" s="64"/>
-      <c r="H12" s="64"/>
-      <c r="I12" s="64" t="s">
+      <c r="G12" s="62"/>
+      <c r="H12" s="62"/>
+      <c r="I12" s="62" t="s">
         <v>10</v>
       </c>
-      <c r="J12" s="64"/>
+      <c r="J12" s="62"/>
       <c r="K12" s="26"/>
     </row>
     <row r="13" spans="1:11" ht="25.05" customHeight="1" x14ac:dyDescent="0.25">
@@ -2125,23 +2101,23 @@
     </row>
     <row r="14" spans="1:11" ht="70.05" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="38"/>
-      <c r="B14" s="86"/>
+      <c r="B14" s="83"/>
       <c r="C14" s="39"/>
-      <c r="D14" s="87"/>
-      <c r="E14" s="86"/>
+      <c r="D14" s="84"/>
+      <c r="E14" s="83"/>
       <c r="F14" s="39"/>
       <c r="G14" s="38"/>
-      <c r="H14" s="86"/>
-      <c r="I14" s="86"/>
+      <c r="H14" s="83"/>
+      <c r="I14" s="83"/>
       <c r="J14" s="38"/>
       <c r="K14" s="39"/>
     </row>
     <row r="15" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="91" t="s">
+      <c r="A15" s="88" t="s">
         <v>15</v>
       </c>
-      <c r="B15" s="92"/>
-      <c r="C15" s="93"/>
+      <c r="B15" s="89"/>
+      <c r="C15" s="90"/>
       <c r="D15" s="50" t="s">
         <v>16</v>
       </c>
@@ -2154,18 +2130,18 @@
       <c r="K15" s="52"/>
     </row>
     <row r="16" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="94"/>
-      <c r="B16" s="95"/>
-      <c r="C16" s="96"/>
-      <c r="D16" s="88" t="s">
+      <c r="A16" s="91"/>
+      <c r="B16" s="92"/>
+      <c r="C16" s="93"/>
+      <c r="D16" s="85" t="s">
         <v>17</v>
       </c>
-      <c r="E16" s="89"/>
-      <c r="F16" s="88" t="s">
+      <c r="E16" s="86"/>
+      <c r="F16" s="85" t="s">
         <v>18</v>
       </c>
-      <c r="G16" s="90"/>
-      <c r="H16" s="89"/>
+      <c r="G16" s="87"/>
+      <c r="H16" s="86"/>
       <c r="I16" s="47" t="s">
         <v>19</v>
       </c>
@@ -2173,16 +2149,16 @@
       <c r="K16" s="49"/>
     </row>
     <row r="17" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="85"/>
-      <c r="B17" s="84"/>
+      <c r="A17" s="82"/>
+      <c r="B17" s="81"/>
       <c r="C17" s="41"/>
       <c r="D17" s="40"/>
       <c r="E17" s="41"/>
       <c r="F17" s="40"/>
-      <c r="G17" s="84"/>
+      <c r="G17" s="81"/>
       <c r="H17" s="41"/>
       <c r="I17" s="40"/>
-      <c r="J17" s="84"/>
+      <c r="J17" s="81"/>
       <c r="K17" s="41"/>
     </row>
     <row r="18" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
@@ -2198,33 +2174,33 @@
       <c r="H18" s="43"/>
       <c r="I18" s="43"/>
       <c r="J18" s="43"/>
-      <c r="K18" s="83"/>
+      <c r="K18" s="80"/>
     </row>
     <row r="19" spans="1:11" ht="70.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="80"/>
-      <c r="B19" s="80"/>
-      <c r="C19" s="80"/>
-      <c r="D19" s="80"/>
-      <c r="E19" s="80"/>
-      <c r="F19" s="80"/>
-      <c r="G19" s="80"/>
-      <c r="H19" s="80"/>
-      <c r="I19" s="80"/>
-      <c r="J19" s="80"/>
-      <c r="K19" s="80"/>
+      <c r="A19" s="75"/>
+      <c r="B19" s="75"/>
+      <c r="C19" s="75"/>
+      <c r="D19" s="75"/>
+      <c r="E19" s="75"/>
+      <c r="F19" s="75"/>
+      <c r="G19" s="75"/>
+      <c r="H19" s="75"/>
+      <c r="I19" s="75"/>
+      <c r="J19" s="75"/>
+      <c r="K19" s="75"/>
     </row>
     <row r="20" spans="1:11" ht="70.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A20" s="81"/>
-      <c r="B20" s="81"/>
-      <c r="C20" s="81"/>
-      <c r="D20" s="81"/>
-      <c r="E20" s="81"/>
-      <c r="F20" s="81"/>
-      <c r="G20" s="81"/>
-      <c r="H20" s="81"/>
-      <c r="I20" s="81"/>
-      <c r="J20" s="81"/>
-      <c r="K20" s="81"/>
+      <c r="A20" s="76"/>
+      <c r="B20" s="76"/>
+      <c r="C20" s="76"/>
+      <c r="D20" s="76"/>
+      <c r="E20" s="76"/>
+      <c r="F20" s="76"/>
+      <c r="G20" s="76"/>
+      <c r="H20" s="76"/>
+      <c r="I20" s="76"/>
+      <c r="J20" s="76"/>
+      <c r="K20" s="76"/>
     </row>
     <row r="21" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="42" t="s">
@@ -2241,17 +2217,17 @@
       <c r="H21" s="43"/>
       <c r="I21" s="43"/>
       <c r="J21" s="43"/>
-      <c r="K21" s="36"/>
+      <c r="K21" s="33"/>
     </row>
     <row r="22" spans="1:11" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="61" t="s">
+      <c r="A22" s="59" t="s">
         <v>23</v>
       </c>
-      <c r="B22" s="62"/>
-      <c r="C22" s="61" t="s">
+      <c r="B22" s="60"/>
+      <c r="C22" s="59" t="s">
         <v>24</v>
       </c>
-      <c r="D22" s="62"/>
+      <c r="D22" s="60"/>
       <c r="E22" s="27" t="s">
         <v>25</v>
       </c>
@@ -2267,159 +2243,159 @@
       <c r="I22" s="27" t="s">
         <v>29</v>
       </c>
-      <c r="J22" s="33" t="s">
+      <c r="J22" s="31" t="s">
         <v>106</v>
       </c>
-      <c r="K22" s="33" t="s">
+      <c r="K22" s="31" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="23" spans="1:11" ht="286.5" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" ht="286.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="53"/>
       <c r="B23" s="54"/>
       <c r="C23" s="38"/>
       <c r="D23" s="39"/>
-      <c r="E23" s="30"/>
-      <c r="F23" s="126"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-      <c r="J23" s="34"/>
-      <c r="K23" s="34"/>
+      <c r="E23" s="35"/>
+      <c r="F23" s="124"/>
+      <c r="G23" s="35"/>
+      <c r="H23" s="35"/>
+      <c r="I23" s="35"/>
+      <c r="J23" s="36"/>
+      <c r="K23" s="36"/>
     </row>
     <row r="24" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="38"/>
       <c r="B24" s="39"/>
       <c r="C24" s="38"/>
       <c r="D24" s="39"/>
-      <c r="E24" s="30"/>
-      <c r="F24" s="127"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
-      <c r="I24" s="30"/>
-      <c r="J24" s="34"/>
-      <c r="K24" s="34"/>
+      <c r="E24" s="35"/>
+      <c r="F24" s="35"/>
+      <c r="G24" s="35"/>
+      <c r="H24" s="35"/>
+      <c r="I24" s="35"/>
+      <c r="J24" s="36"/>
+      <c r="K24" s="36"/>
     </row>
     <row r="25" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="38"/>
       <c r="B25" s="39"/>
       <c r="C25" s="38"/>
       <c r="D25" s="39"/>
-      <c r="E25" s="30"/>
-      <c r="F25" s="127"/>
-      <c r="G25" s="30"/>
-      <c r="H25" s="30"/>
-      <c r="I25" s="30"/>
-      <c r="J25" s="34"/>
-      <c r="K25" s="34"/>
+      <c r="E25" s="35"/>
+      <c r="F25" s="35"/>
+      <c r="G25" s="35"/>
+      <c r="H25" s="35"/>
+      <c r="I25" s="35"/>
+      <c r="J25" s="36"/>
+      <c r="K25" s="36"/>
     </row>
     <row r="26" spans="1:11" ht="210" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="38"/>
       <c r="B26" s="39"/>
       <c r="C26" s="38"/>
       <c r="D26" s="39"/>
-      <c r="E26" s="30"/>
-      <c r="F26" s="127"/>
-      <c r="G26" s="30"/>
-      <c r="H26" s="30"/>
-      <c r="I26" s="30"/>
-      <c r="J26" s="34"/>
-      <c r="K26" s="34"/>
+      <c r="E26" s="35"/>
+      <c r="F26" s="35"/>
+      <c r="G26" s="35"/>
+      <c r="H26" s="35"/>
+      <c r="I26" s="35"/>
+      <c r="J26" s="36"/>
+      <c r="K26" s="36"/>
     </row>
     <row r="27" spans="1:11" ht="210" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A27" s="40"/>
       <c r="B27" s="41"/>
       <c r="C27" s="40"/>
       <c r="D27" s="41"/>
-      <c r="E27" s="31"/>
-      <c r="F27" s="128"/>
-      <c r="G27" s="31"/>
-      <c r="H27" s="31"/>
-      <c r="I27" s="31"/>
-      <c r="J27" s="34"/>
-      <c r="K27" s="34"/>
+      <c r="E27" s="37"/>
+      <c r="F27" s="37"/>
+      <c r="G27" s="37"/>
+      <c r="H27" s="37"/>
+      <c r="I27" s="37"/>
+      <c r="J27" s="36"/>
+      <c r="K27" s="36"/>
     </row>
     <row r="28" spans="1:11" s="18" customFormat="1" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A28" s="66" t="s">
+      <c r="A28" s="77" t="s">
         <v>30</v>
       </c>
-      <c r="B28" s="67"/>
-      <c r="C28" s="67"/>
-      <c r="D28" s="67"/>
-      <c r="E28" s="67"/>
-      <c r="F28" s="67"/>
-      <c r="G28" s="67"/>
-      <c r="H28" s="67"/>
-      <c r="I28" s="67"/>
-      <c r="J28" s="68"/>
-      <c r="K28" s="69"/>
+      <c r="B28" s="78"/>
+      <c r="C28" s="78"/>
+      <c r="D28" s="78"/>
+      <c r="E28" s="78"/>
+      <c r="F28" s="78"/>
+      <c r="G28" s="78"/>
+      <c r="H28" s="78"/>
+      <c r="I28" s="78"/>
+      <c r="J28" s="104"/>
+      <c r="K28" s="105"/>
     </row>
     <row r="29" spans="1:11" ht="70.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="110"/>
-      <c r="B29" s="110"/>
-      <c r="C29" s="110"/>
-      <c r="D29" s="110"/>
-      <c r="E29" s="110"/>
-      <c r="F29" s="110"/>
-      <c r="G29" s="110"/>
-      <c r="H29" s="110"/>
-      <c r="I29" s="110"/>
-      <c r="J29" s="110"/>
-      <c r="K29" s="110"/>
+      <c r="A29" s="111"/>
+      <c r="B29" s="111"/>
+      <c r="C29" s="111"/>
+      <c r="D29" s="111"/>
+      <c r="E29" s="111"/>
+      <c r="F29" s="111"/>
+      <c r="G29" s="111"/>
+      <c r="H29" s="111"/>
+      <c r="I29" s="111"/>
+      <c r="J29" s="111"/>
+      <c r="K29" s="111"/>
     </row>
     <row r="30" spans="1:11" ht="70.05" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A30" s="111"/>
-      <c r="B30" s="111"/>
-      <c r="C30" s="111"/>
-      <c r="D30" s="111"/>
-      <c r="E30" s="111"/>
-      <c r="F30" s="111"/>
-      <c r="G30" s="111"/>
-      <c r="H30" s="111"/>
-      <c r="I30" s="111"/>
-      <c r="J30" s="111"/>
-      <c r="K30" s="111"/>
+      <c r="A30" s="112"/>
+      <c r="B30" s="112"/>
+      <c r="C30" s="112"/>
+      <c r="D30" s="112"/>
+      <c r="E30" s="112"/>
+      <c r="F30" s="112"/>
+      <c r="G30" s="112"/>
+      <c r="H30" s="112"/>
+      <c r="I30" s="112"/>
+      <c r="J30" s="112"/>
+      <c r="K30" s="112"/>
     </row>
     <row r="31" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A31" s="66" t="s">
+      <c r="A31" s="77" t="s">
         <v>31</v>
       </c>
-      <c r="B31" s="67"/>
-      <c r="C31" s="67"/>
-      <c r="D31" s="67"/>
-      <c r="E31" s="67"/>
-      <c r="F31" s="67"/>
-      <c r="G31" s="67"/>
-      <c r="H31" s="67"/>
-      <c r="I31" s="67"/>
-      <c r="J31" s="67"/>
-      <c r="K31" s="82"/>
+      <c r="B31" s="78"/>
+      <c r="C31" s="78"/>
+      <c r="D31" s="78"/>
+      <c r="E31" s="78"/>
+      <c r="F31" s="78"/>
+      <c r="G31" s="78"/>
+      <c r="H31" s="78"/>
+      <c r="I31" s="78"/>
+      <c r="J31" s="78"/>
+      <c r="K31" s="79"/>
     </row>
     <row r="32" spans="1:11" ht="70.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="104"/>
-      <c r="B32" s="105"/>
-      <c r="C32" s="105"/>
-      <c r="D32" s="105"/>
-      <c r="E32" s="105"/>
-      <c r="F32" s="105"/>
-      <c r="G32" s="105"/>
-      <c r="H32" s="105"/>
-      <c r="I32" s="105"/>
-      <c r="J32" s="105"/>
-      <c r="K32" s="106"/>
+      <c r="A32" s="107"/>
+      <c r="B32" s="108"/>
+      <c r="C32" s="108"/>
+      <c r="D32" s="108"/>
+      <c r="E32" s="108"/>
+      <c r="F32" s="108"/>
+      <c r="G32" s="108"/>
+      <c r="H32" s="108"/>
+      <c r="I32" s="108"/>
+      <c r="J32" s="108"/>
+      <c r="K32" s="109"/>
     </row>
     <row r="33" spans="1:11" ht="70.05" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="107"/>
-      <c r="B33" s="108"/>
-      <c r="C33" s="108"/>
-      <c r="D33" s="108"/>
-      <c r="E33" s="108"/>
-      <c r="F33" s="108"/>
-      <c r="G33" s="108"/>
-      <c r="H33" s="108"/>
-      <c r="I33" s="108"/>
-      <c r="J33" s="108"/>
-      <c r="K33" s="109"/>
+      <c r="A33" s="102"/>
+      <c r="B33" s="110"/>
+      <c r="C33" s="110"/>
+      <c r="D33" s="110"/>
+      <c r="E33" s="110"/>
+      <c r="F33" s="110"/>
+      <c r="G33" s="110"/>
+      <c r="H33" s="110"/>
+      <c r="I33" s="110"/>
+      <c r="J33" s="110"/>
+      <c r="K33" s="103"/>
     </row>
     <row r="34" spans="1:11" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="19" t="s">
@@ -2434,7 +2410,7 @@
       <c r="H34" s="20"/>
       <c r="I34" s="20"/>
       <c r="J34" s="20"/>
-      <c r="K34" s="103"/>
+      <c r="K34" s="106"/>
     </row>
     <row r="35" spans="1:11" ht="20.100000000000001" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A35" s="28" t="s">
@@ -2449,56 +2425,56 @@
       <c r="H35" s="29"/>
       <c r="I35" s="29"/>
       <c r="J35" s="29"/>
-      <c r="K35" s="103"/>
+      <c r="K35" s="106"/>
     </row>
     <row r="36" spans="1:11" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A36" s="66" t="s">
+      <c r="A36" s="77" t="s">
         <v>34</v>
       </c>
-      <c r="B36" s="67"/>
-      <c r="C36" s="67"/>
-      <c r="D36" s="67"/>
-      <c r="E36" s="67"/>
-      <c r="F36" s="67"/>
-      <c r="G36" s="67"/>
-      <c r="H36" s="67"/>
-      <c r="I36" s="67"/>
-      <c r="J36" s="67"/>
-      <c r="K36" s="82"/>
+      <c r="B36" s="78"/>
+      <c r="C36" s="78"/>
+      <c r="D36" s="78"/>
+      <c r="E36" s="78"/>
+      <c r="F36" s="78"/>
+      <c r="G36" s="78"/>
+      <c r="H36" s="78"/>
+      <c r="I36" s="78"/>
+      <c r="J36" s="78"/>
+      <c r="K36" s="79"/>
     </row>
     <row r="37" spans="1:11" ht="35.1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="123" t="s">
+      <c r="A37" s="96" t="s">
         <v>38</v>
       </c>
-      <c r="B37" s="124"/>
-      <c r="C37" s="124"/>
-      <c r="D37" s="125"/>
-      <c r="E37" s="98" t="s">
+      <c r="B37" s="97"/>
+      <c r="C37" s="97"/>
+      <c r="D37" s="98"/>
+      <c r="E37" s="99" t="s">
         <v>36</v>
       </c>
-      <c r="F37" s="98"/>
-      <c r="G37" s="98"/>
-      <c r="H37" s="99" t="s">
+      <c r="F37" s="99"/>
+      <c r="G37" s="99"/>
+      <c r="H37" s="100" t="s">
         <v>37</v>
       </c>
-      <c r="I37" s="100"/>
-      <c r="J37" s="101" t="s">
+      <c r="I37" s="101"/>
+      <c r="J37" s="102" t="s">
         <v>35</v>
       </c>
-      <c r="K37" s="102"/>
+      <c r="K37" s="103"/>
     </row>
   </sheetData>
   <mergeCells count="56">
+    <mergeCell ref="A37:D37"/>
+    <mergeCell ref="E37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="A28:K28"/>
     <mergeCell ref="K34:K35"/>
     <mergeCell ref="A32:K33"/>
     <mergeCell ref="A31:K31"/>
     <mergeCell ref="A29:K30"/>
     <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A37:D37"/>
-    <mergeCell ref="E37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="A28:K28"/>
     <mergeCell ref="A1:A6"/>
     <mergeCell ref="B1:K2"/>
     <mergeCell ref="A19:K20"/>
@@ -2607,20 +2583,20 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="120" t="s">
+      <c r="B2" s="121" t="s">
         <v>39</v>
       </c>
-      <c r="C2" s="120"/>
-      <c r="D2" s="120"/>
-      <c r="E2" s="120"/>
-      <c r="F2" s="120"/>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
-      <c r="M2" s="120"/>
+      <c r="C2" s="121"/>
+      <c r="D2" s="121"/>
+      <c r="E2" s="121"/>
+      <c r="F2" s="121"/>
+      <c r="G2" s="121"/>
+      <c r="H2" s="121"/>
+      <c r="I2" s="121"/>
+      <c r="J2" s="121"/>
+      <c r="K2" s="121"/>
+      <c r="L2" s="121"/>
+      <c r="M2" s="121"/>
     </row>
     <row r="3" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="2"/>
@@ -2652,21 +2628,21 @@
     </row>
     <row r="5" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.3"/>
     <row r="6" spans="2:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="119" t="s">
+      <c r="B6" s="120" t="s">
         <v>40</v>
       </c>
-      <c r="C6" s="119"/>
-      <c r="D6" s="119"/>
-      <c r="E6" s="119"/>
-      <c r="G6" s="119" t="s">
+      <c r="C6" s="120"/>
+      <c r="D6" s="120"/>
+      <c r="E6" s="120"/>
+      <c r="G6" s="120" t="s">
         <v>41</v>
       </c>
-      <c r="H6" s="119"/>
-      <c r="I6" s="119"/>
-      <c r="J6" s="119"/>
-      <c r="K6" s="119"/>
-      <c r="L6" s="119"/>
-      <c r="M6" s="119"/>
+      <c r="H6" s="120"/>
+      <c r="I6" s="120"/>
+      <c r="J6" s="120"/>
+      <c r="K6" s="120"/>
+      <c r="L6" s="120"/>
+      <c r="M6" s="120"/>
     </row>
     <row r="7" spans="2:13" ht="12.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="3"/>
@@ -2708,7 +2684,7 @@
       <c r="E9" s="8" t="s">
         <v>49</v>
       </c>
-      <c r="G9" s="121" t="s">
+      <c r="G9" s="122" t="s">
         <v>50</v>
       </c>
       <c r="H9" s="7" t="s">
@@ -2743,7 +2719,7 @@
       <c r="E10" s="8" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="121"/>
+      <c r="G10" s="122"/>
       <c r="H10" s="7" t="s">
         <v>56</v>
       </c>
@@ -2776,7 +2752,7 @@
       <c r="E11" s="8" t="s">
         <v>60</v>
       </c>
-      <c r="G11" s="121"/>
+      <c r="G11" s="122"/>
       <c r="H11" s="7" t="s">
         <v>61</v>
       </c>
@@ -2809,7 +2785,7 @@
       <c r="E12" s="8" t="s">
         <v>65</v>
       </c>
-      <c r="G12" s="121"/>
+      <c r="G12" s="122"/>
       <c r="H12" s="7" t="s">
         <v>66</v>
       </c>
@@ -2842,7 +2818,7 @@
       <c r="E13" s="8" t="s">
         <v>70</v>
       </c>
-      <c r="G13" s="121"/>
+      <c r="G13" s="122"/>
       <c r="H13" s="7" t="s">
         <v>71</v>
       </c>
@@ -2880,30 +2856,30 @@
       </c>
     </row>
     <row r="15" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="I15" s="122" t="s">
+      <c r="I15" s="123" t="s">
         <v>77</v>
       </c>
-      <c r="J15" s="122"/>
-      <c r="K15" s="122"/>
-      <c r="L15" s="122"/>
-      <c r="M15" s="122"/>
+      <c r="J15" s="123"/>
+      <c r="K15" s="123"/>
+      <c r="L15" s="123"/>
+      <c r="M15" s="123"/>
     </row>
     <row r="19" spans="2:13" ht="20.100000000000001" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="119" t="s">
+      <c r="B19" s="120" t="s">
         <v>78</v>
       </c>
-      <c r="C19" s="119"/>
-      <c r="D19" s="119"/>
-      <c r="E19" s="119"/>
-      <c r="G19" s="119" t="s">
+      <c r="C19" s="120"/>
+      <c r="D19" s="120"/>
+      <c r="E19" s="120"/>
+      <c r="G19" s="120" t="s">
         <v>79</v>
       </c>
-      <c r="H19" s="119"/>
-      <c r="I19" s="119"/>
-      <c r="J19" s="119"/>
-      <c r="K19" s="119"/>
-      <c r="L19" s="119"/>
-      <c r="M19" s="119"/>
+      <c r="H19" s="120"/>
+      <c r="I19" s="120"/>
+      <c r="J19" s="120"/>
+      <c r="K19" s="120"/>
+      <c r="L19" s="120"/>
+      <c r="M19" s="120"/>
     </row>
     <row r="21" spans="2:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="4" t="s">
@@ -2912,21 +2888,21 @@
       <c r="C21" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D21" s="116" t="s">
+      <c r="D21" s="117" t="s">
         <v>82</v>
       </c>
-      <c r="E21" s="116"/>
-      <c r="G21" s="117" t="s">
+      <c r="E21" s="117"/>
+      <c r="G21" s="118" t="s">
         <v>83</v>
       </c>
-      <c r="H21" s="117"/>
-      <c r="I21" s="117" t="s">
+      <c r="H21" s="118"/>
+      <c r="I21" s="118" t="s">
         <v>23</v>
       </c>
-      <c r="J21" s="117"/>
-      <c r="K21" s="117"/>
-      <c r="L21" s="117"/>
-      <c r="M21" s="37" t="s">
+      <c r="J21" s="118"/>
+      <c r="K21" s="118"/>
+      <c r="L21" s="118"/>
+      <c r="M21" s="34" t="s">
         <v>107</v>
       </c>
     </row>
@@ -2937,21 +2913,21 @@
       <c r="C22" s="8" t="s">
         <v>85</v>
       </c>
-      <c r="D22" s="113" t="s">
+      <c r="D22" s="114" t="s">
         <v>86</v>
       </c>
-      <c r="E22" s="113"/>
-      <c r="G22" s="118" t="s">
+      <c r="E22" s="114"/>
+      <c r="G22" s="119" t="s">
         <v>87</v>
       </c>
-      <c r="H22" s="118"/>
-      <c r="I22" s="112" t="s">
+      <c r="H22" s="119"/>
+      <c r="I22" s="113" t="s">
         <v>88</v>
       </c>
-      <c r="J22" s="112"/>
-      <c r="K22" s="112"/>
-      <c r="L22" s="112"/>
-      <c r="M22" s="35" t="s">
+      <c r="J22" s="113"/>
+      <c r="K22" s="113"/>
+      <c r="L22" s="113"/>
+      <c r="M22" s="32" t="s">
         <v>108</v>
       </c>
     </row>
@@ -2962,21 +2938,21 @@
       <c r="C23" s="8" t="s">
         <v>90</v>
       </c>
-      <c r="D23" s="113" t="s">
+      <c r="D23" s="114" t="s">
         <v>91</v>
       </c>
-      <c r="E23" s="113"/>
-      <c r="G23" s="114" t="s">
+      <c r="E23" s="114"/>
+      <c r="G23" s="115" t="s">
         <v>92</v>
       </c>
-      <c r="H23" s="114"/>
-      <c r="I23" s="112" t="s">
+      <c r="H23" s="115"/>
+      <c r="I23" s="113" t="s">
         <v>93</v>
       </c>
-      <c r="J23" s="112"/>
-      <c r="K23" s="112"/>
-      <c r="L23" s="112"/>
-      <c r="M23" s="35" t="s">
+      <c r="J23" s="113"/>
+      <c r="K23" s="113"/>
+      <c r="L23" s="113"/>
+      <c r="M23" s="32" t="s">
         <v>109</v>
       </c>
     </row>
@@ -2987,21 +2963,21 @@
       <c r="C24" s="8" t="s">
         <v>95</v>
       </c>
-      <c r="D24" s="113" t="s">
+      <c r="D24" s="114" t="s">
         <v>96</v>
       </c>
-      <c r="E24" s="113"/>
-      <c r="G24" s="115" t="s">
+      <c r="E24" s="114"/>
+      <c r="G24" s="116" t="s">
         <v>97</v>
       </c>
-      <c r="H24" s="115"/>
-      <c r="I24" s="112" t="s">
+      <c r="H24" s="116"/>
+      <c r="I24" s="113" t="s">
         <v>98</v>
       </c>
-      <c r="J24" s="112"/>
-      <c r="K24" s="112"/>
-      <c r="L24" s="112"/>
-      <c r="M24" s="35" t="s">
+      <c r="J24" s="113"/>
+      <c r="K24" s="113"/>
+      <c r="L24" s="113"/>
+      <c r="M24" s="32" t="s">
         <v>110</v>
       </c>
     </row>
@@ -3012,10 +2988,10 @@
       <c r="C25" s="8" t="s">
         <v>100</v>
       </c>
-      <c r="D25" s="113" t="s">
+      <c r="D25" s="114" t="s">
         <v>101</v>
       </c>
-      <c r="E25" s="113"/>
+      <c r="E25" s="114"/>
     </row>
     <row r="26" spans="2:13" ht="50.1" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="7" t="s">
@@ -3024,10 +3000,10 @@
       <c r="C26" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D26" s="113" t="s">
+      <c r="D26" s="114" t="s">
         <v>104</v>
       </c>
-      <c r="E26" s="113"/>
+      <c r="E26" s="114"/>
     </row>
   </sheetData>
   <mergeCells count="21">

</xml_diff>